<commit_message>
feat(seed): align roster xlsx and mock-agent with students fixture
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/scripts/sample-roster-bad.xlsx
+++ b/scripts/sample-roster-bad.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="52">
   <si>
-    <t>DANH SÁCH LỚP — CS101 Nhóm 01</t>
+    <t>DANH SÁCH LỚP — 4220004247 Nhóm 01</t>
   </si>
   <si>
     <t>STT</t>
@@ -28,145 +28,145 @@
     <t>Ghi chú</t>
   </si>
   <si>
-    <t>MSSVTEST01</t>
-  </si>
-  <si>
-    <t>Sinh viên test 01</t>
+    <t>24000301</t>
+  </si>
+  <si>
+    <t>Nguyễn Hoàng Minh</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>MSSVTEST02</t>
-  </si>
-  <si>
-    <t>Sinh viên test 02</t>
-  </si>
-  <si>
-    <t>MSSVTEST03</t>
-  </si>
-  <si>
-    <t>Sinh viên test 03</t>
-  </si>
-  <si>
-    <t>MSSVTEST04</t>
-  </si>
-  <si>
-    <t>Sinh viên test 04</t>
-  </si>
-  <si>
-    <t>MSSVTEST05</t>
-  </si>
-  <si>
-    <t>Sinh viên test 05</t>
-  </si>
-  <si>
-    <t>SV 2012 0003</t>
+    <t>24000302</t>
+  </si>
+  <si>
+    <t>Trần Thị Mai Anh</t>
+  </si>
+  <si>
+    <t>24000303</t>
+  </si>
+  <si>
+    <t>Lê Văn Đức</t>
+  </si>
+  <si>
+    <t>24000304</t>
+  </si>
+  <si>
+    <t>Phạm Thị Thu Hà</t>
+  </si>
+  <si>
+    <t>24000305</t>
+  </si>
+  <si>
+    <t>Hoàng Minh Tuấn</t>
+  </si>
+  <si>
+    <t>240 00399</t>
   </si>
   <si>
     <t>Lê Văn Hỏng</t>
   </si>
   <si>
-    <t>MSSVTEST06</t>
-  </si>
-  <si>
-    <t>Sinh viên test 06</t>
-  </si>
-  <si>
-    <t>MSSVTEST07</t>
-  </si>
-  <si>
-    <t>Sinh viên test 07</t>
-  </si>
-  <si>
-    <t>MSSVTEST08</t>
-  </si>
-  <si>
-    <t>Sinh viên test 08</t>
-  </si>
-  <si>
-    <t>MSSVTEST09</t>
-  </si>
-  <si>
-    <t>Sinh viên test 09</t>
-  </si>
-  <si>
-    <t>MSSVTEST10</t>
-  </si>
-  <si>
-    <t>Sinh viên test 10</t>
-  </si>
-  <si>
-    <t>MSSVTEST11</t>
-  </si>
-  <si>
-    <t>Sinh viên test 11</t>
-  </si>
-  <si>
-    <t>MSSVTEST12</t>
-  </si>
-  <si>
-    <t>Sinh viên test 12</t>
-  </si>
-  <si>
-    <t>MSSVTEST13</t>
-  </si>
-  <si>
-    <t>Sinh viên test 13</t>
-  </si>
-  <si>
-    <t>MSSVTEST14</t>
-  </si>
-  <si>
-    <t>Sinh viên test 14</t>
-  </si>
-  <si>
-    <t>MSSVTEST15</t>
-  </si>
-  <si>
-    <t>Sinh viên test 15</t>
-  </si>
-  <si>
-    <t>MSSVTEST16</t>
-  </si>
-  <si>
-    <t>Sinh viên test 16</t>
-  </si>
-  <si>
-    <t>MSSVTEST17</t>
-  </si>
-  <si>
-    <t>Sinh viên test 17</t>
-  </si>
-  <si>
-    <t>MSSVTEST18</t>
-  </si>
-  <si>
-    <t>Sinh viên test 18</t>
-  </si>
-  <si>
-    <t>MSSVTEST19</t>
-  </si>
-  <si>
-    <t>Sinh viên test 19</t>
-  </si>
-  <si>
-    <t>MSSVTEST20</t>
-  </si>
-  <si>
-    <t>Sinh viên test 20</t>
-  </si>
-  <si>
-    <t>SV20120001</t>
-  </si>
-  <si>
-    <t>Nguyễn Văn A</t>
-  </si>
-  <si>
-    <t>SV20120002</t>
-  </si>
-  <si>
-    <t>Trần Thị B</t>
+    <t>24000306</t>
+  </si>
+  <si>
+    <t>Võ Thị Kim Ngân</t>
+  </si>
+  <si>
+    <t>24000307</t>
+  </si>
+  <si>
+    <t>Đặng Quốc Bảo</t>
+  </si>
+  <si>
+    <t>24000308</t>
+  </si>
+  <si>
+    <t>Bùi Thị Lan Hương</t>
+  </si>
+  <si>
+    <t>24000309</t>
+  </si>
+  <si>
+    <t>Ngô Văn Khoa</t>
+  </si>
+  <si>
+    <t>24000310</t>
+  </si>
+  <si>
+    <t>Đỗ Thị Thanh Trúc</t>
+  </si>
+  <si>
+    <t>24000311</t>
+  </si>
+  <si>
+    <t>Phan Anh Dũng</t>
+  </si>
+  <si>
+    <t>24000312</t>
+  </si>
+  <si>
+    <t>Lý Thị Mỹ Linh</t>
+  </si>
+  <si>
+    <t>24000313</t>
+  </si>
+  <si>
+    <t>Trương Nhật Nam</t>
+  </si>
+  <si>
+    <t>24000314</t>
+  </si>
+  <si>
+    <t>Huỳnh Thị Ngọc Diễm</t>
+  </si>
+  <si>
+    <t>24000315</t>
+  </si>
+  <si>
+    <t>Cao Văn Phúc</t>
+  </si>
+  <si>
+    <t>24000316</t>
+  </si>
+  <si>
+    <t>Đinh Thị Hồng Nhung</t>
+  </si>
+  <si>
+    <t>24000317</t>
+  </si>
+  <si>
+    <t>Mai Quốc Huy</t>
+  </si>
+  <si>
+    <t>24000318</t>
+  </si>
+  <si>
+    <t>Tạ Thị Phương Thảo</t>
+  </si>
+  <si>
+    <t>24000319</t>
+  </si>
+  <si>
+    <t>Lâm Văn Sơn</t>
+  </si>
+  <si>
+    <t>24000320</t>
+  </si>
+  <si>
+    <t>Châu Thị Bảo Yến</t>
+  </si>
+  <si>
+    <t>24000321</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn An</t>
+  </si>
+  <si>
+    <t>24000322</t>
+  </si>
+  <si>
+    <t>Trần Thị Bình</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat(web): harden roster import and catalog student add
Support richer Excel mapping, export nominal-class students, and pick catalog students when adding to roster.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/scripts/sample-roster-bad.xlsx
+++ b/scripts/sample-roster-bad.xlsx
@@ -28,7 +28,7 @@
     <t>Ghi chú</t>
   </si>
   <si>
-    <t>MSSVTEST01</t>
+    <t>20000001</t>
   </si>
   <si>
     <t>Sinh viên test 01</t>
@@ -37,25 +37,25 @@
     <t/>
   </si>
   <si>
-    <t>MSSVTEST02</t>
+    <t>20000002</t>
   </si>
   <si>
     <t>Sinh viên test 02</t>
   </si>
   <si>
-    <t>MSSVTEST03</t>
+    <t>20000003</t>
   </si>
   <si>
     <t>Sinh viên test 03</t>
   </si>
   <si>
-    <t>MSSVTEST04</t>
+    <t>20000004</t>
   </si>
   <si>
     <t>Sinh viên test 04</t>
   </si>
   <si>
-    <t>MSSVTEST05</t>
+    <t>20000005</t>
   </si>
   <si>
     <t>Sinh viên test 05</t>
@@ -67,103 +67,103 @@
     <t>Lê Văn Hỏng</t>
   </si>
   <si>
-    <t>MSSVTEST06</t>
+    <t>20000006</t>
   </si>
   <si>
     <t>Sinh viên test 06</t>
   </si>
   <si>
-    <t>MSSVTEST07</t>
+    <t>20000007</t>
   </si>
   <si>
     <t>Sinh viên test 07</t>
   </si>
   <si>
-    <t>MSSVTEST08</t>
+    <t>20000008</t>
   </si>
   <si>
     <t>Sinh viên test 08</t>
   </si>
   <si>
-    <t>MSSVTEST09</t>
+    <t>20000009</t>
   </si>
   <si>
     <t>Sinh viên test 09</t>
   </si>
   <si>
-    <t>MSSVTEST10</t>
+    <t>20000010</t>
   </si>
   <si>
     <t>Sinh viên test 10</t>
   </si>
   <si>
-    <t>MSSVTEST11</t>
+    <t>20000011</t>
   </si>
   <si>
     <t>Sinh viên test 11</t>
   </si>
   <si>
-    <t>MSSVTEST12</t>
+    <t>20000012</t>
   </si>
   <si>
     <t>Sinh viên test 12</t>
   </si>
   <si>
-    <t>MSSVTEST13</t>
+    <t>20000013</t>
   </si>
   <si>
     <t>Sinh viên test 13</t>
   </si>
   <si>
-    <t>MSSVTEST14</t>
+    <t>20000014</t>
   </si>
   <si>
     <t>Sinh viên test 14</t>
   </si>
   <si>
-    <t>MSSVTEST15</t>
+    <t>20000015</t>
   </si>
   <si>
     <t>Sinh viên test 15</t>
   </si>
   <si>
-    <t>MSSVTEST16</t>
+    <t>20000016</t>
   </si>
   <si>
     <t>Sinh viên test 16</t>
   </si>
   <si>
-    <t>MSSVTEST17</t>
+    <t>20000017</t>
   </si>
   <si>
     <t>Sinh viên test 17</t>
   </si>
   <si>
-    <t>MSSVTEST18</t>
+    <t>20000018</t>
   </si>
   <si>
     <t>Sinh viên test 18</t>
   </si>
   <si>
-    <t>MSSVTEST19</t>
+    <t>20000019</t>
   </si>
   <si>
     <t>Sinh viên test 19</t>
   </si>
   <si>
-    <t>MSSVTEST20</t>
+    <t>20000020</t>
   </si>
   <si>
     <t>Sinh viên test 20</t>
   </si>
   <si>
-    <t>SV20120001</t>
+    <t>20120001</t>
   </si>
   <si>
     <t>Nguyễn Văn A</t>
   </si>
   <si>
-    <t>SV20120002</t>
+    <t>20120002</t>
   </si>
   <si>
     <t>Trần Thị B</t>

</xml_diff>